<commit_message>
final improvements: highlighting, parallax depth field, node inspector, pinning
</commit_message>
<xml_diff>
--- a/time_tracking.xlsx
+++ b/time_tracking.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maxim/UCLL/Jaar 3/Sem 2/Research &amp; Expertise Project Digital Solutions/Interactive-3D-Force-Directed-Graph-Visualization/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06C95256-516B-EF44-AAEA-FC0A23241900}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7A1EA45-9664-2E4F-AE86-234621F6B032}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>Date</t>
   </si>
@@ -44,6 +44,9 @@
     <t>Hours</t>
   </si>
   <si>
+    <t>Kick off / `planning</t>
+  </si>
+  <si>
     <t>Initial commit: repository setup, branching strategy</t>
   </si>
   <si>
@@ -53,9 +56,39 @@
     <t>Project scaffold: Express server, client folder, config files, README</t>
   </si>
   <si>
+    <t>Research</t>
+  </si>
+  <si>
+    <t>Research: 3d-force-graph library</t>
+  </si>
+  <si>
+    <t>Research: CouchDB</t>
+  </si>
+  <si>
+    <t>Research: CORDIS Horizon dataset</t>
+  </si>
+  <si>
+    <t>CouchDB installation, admin user creation, CORS config</t>
+  </si>
+  <si>
+    <t>Research: D3 force simulation</t>
+  </si>
+  <si>
+    <t>CouchDB document schema</t>
+  </si>
+  <si>
+    <t>Node.js async/await patterns, Express 5 routing, fetch API</t>
+  </si>
+  <si>
+    <t>Development</t>
+  </si>
+  <si>
     <t>CouchDB import script design, couchdb-setup.md documentation (c2e96dd)</t>
   </si>
   <si>
+    <t>feat: Excel -&gt; CouchDB import script + inspect tool; added xlsx + minimist deps</t>
+  </si>
+  <si>
     <t>Testing import script: dry run, debugging field mappings, running full import</t>
   </si>
   <si>
@@ -113,57 +146,28 @@
     <t>cleanup/fix: duplicate function declarations, inconsistent variable names, CSS</t>
   </si>
   <si>
-    <t>Research</t>
-  </si>
-  <si>
-    <t>Development</t>
-  </si>
-  <si>
-    <t>feat: Excel -&gt; CouchDB import script + inspect tool; added xlsx + minimist deps</t>
+    <t>Refactor: improved structure to better explore the code for grading</t>
+  </si>
+  <si>
+    <t>Fix(ui): improved the controls panel</t>
+  </si>
+  <si>
+    <t>Styling improvement for visibility, glowing fix + GLTF</t>
   </si>
   <si>
     <t>totaal:</t>
   </si>
   <si>
-    <t>Kick off / `planning</t>
-  </si>
-  <si>
-    <t>Refactor: improved structure to better explore the code for grading</t>
-  </si>
-  <si>
-    <t>Research: 3d-force-graph library</t>
-  </si>
-  <si>
-    <t>Research: CouchDB</t>
-  </si>
-  <si>
-    <t>Research: CORDIS Horizon dataset</t>
-  </si>
-  <si>
-    <t>Fix(ui): improved the controls panel</t>
-  </si>
-  <si>
-    <t>CouchDB installation, admin user creation, CORS config</t>
-  </si>
-  <si>
-    <t>Research: D3 force simulation</t>
-  </si>
-  <si>
-    <t>CouchDB document schema</t>
-  </si>
-  <si>
-    <t>Node.js async/await patterns, Express 5 routing, fetch API</t>
-  </si>
-  <si>
-    <t>Styling improvement for visibility, glowing fix + GLTF</t>
+    <t>fix(modules): duplicate export, missing imports, GLTFLoader importmap, script load order</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="d/mm/yyyy;@"/>
+    <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -314,7 +318,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -369,6 +373,12 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -672,7 +682,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -693,7 +703,7 @@
     </row>
     <row r="2" spans="1:3" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="13" t="s">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="B2" s="14"/>
       <c r="C2" s="15"/>
@@ -703,7 +713,7 @@
         <v>46136</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C3" s="1">
         <v>1</v>
@@ -714,7 +724,7 @@
         <v>46137</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C4" s="3">
         <v>0.5</v>
@@ -725,7 +735,7 @@
         <v>46139</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C5" s="1">
         <v>2</v>
@@ -733,7 +743,7 @@
     </row>
     <row r="6" spans="1:3" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="13" t="s">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="B6" s="14"/>
       <c r="C6" s="15"/>
@@ -743,7 +753,7 @@
         <v>46140</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C7" s="1">
         <v>2.5</v>
@@ -754,7 +764,7 @@
         <v>46141</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="C8" s="3">
         <v>2</v>
@@ -765,7 +775,7 @@
         <v>46142</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="C9" s="1">
         <v>0.75</v>
@@ -776,7 +786,7 @@
         <v>46146</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="C10" s="3">
         <v>2.5</v>
@@ -787,7 +797,7 @@
         <v>46147</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="C11" s="1">
         <v>2</v>
@@ -798,7 +808,7 @@
         <v>46148</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="C12" s="3">
         <v>1</v>
@@ -809,7 +819,7 @@
         <v>46149</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>39</v>
+        <v>14</v>
       </c>
       <c r="C13" s="1">
         <v>0.5</v>
@@ -817,7 +827,7 @@
     </row>
     <row r="14" spans="1:3" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="13" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -827,7 +837,7 @@
         <v>46154</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="C15" s="1">
         <v>3</v>
@@ -838,7 +848,7 @@
         <v>46155</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="C16" s="3">
         <v>3.5</v>
@@ -849,7 +859,7 @@
         <v>46156</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="C17" s="1">
         <v>2.5</v>
@@ -860,7 +870,7 @@
         <v>46157</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="C18" s="3">
         <v>3</v>
@@ -871,7 +881,7 @@
         <v>46160</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="C19" s="6">
         <v>3</v>
@@ -882,7 +892,7 @@
         <v>46161</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="C20" s="3">
         <v>1.5</v>
@@ -893,7 +903,7 @@
         <v>46162</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="C21" s="6">
         <v>4.5</v>
@@ -904,7 +914,7 @@
         <v>46163</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="C22" s="3">
         <v>2</v>
@@ -915,7 +925,7 @@
         <v>46168</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="C23" s="1">
         <v>1</v>
@@ -926,7 +936,7 @@
         <v>46169</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="C24" s="3">
         <v>5.5</v>
@@ -937,7 +947,7 @@
         <v>46170</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="C25" s="6">
         <v>4</v>
@@ -948,7 +958,7 @@
         <v>46171</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="C26" s="3">
         <v>3</v>
@@ -959,7 +969,7 @@
         <v>46172</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="C27" s="6">
         <v>1.5</v>
@@ -970,7 +980,7 @@
         <v>46174</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="C28" s="3">
         <v>2</v>
@@ -981,7 +991,7 @@
         <v>46176</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="C29" s="1">
         <v>1.5</v>
@@ -992,7 +1002,7 @@
         <v>46179</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="C30" s="3">
         <v>2.5</v>
@@ -1003,7 +1013,7 @@
         <v>46180</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="C31" s="1">
         <v>2</v>
@@ -1014,7 +1024,7 @@
         <v>46181</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="C32" s="3">
         <v>4.5</v>
@@ -1025,7 +1035,7 @@
         <v>46182</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="C33" s="1">
         <v>2</v>
@@ -1036,7 +1046,7 @@
         <v>46183</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="C34" s="3">
         <v>2</v>
@@ -1047,7 +1057,7 @@
         <v>46183</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="C35" s="6">
         <v>3.5</v>
@@ -1058,7 +1068,7 @@
         <v>46187</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="C36" s="12">
         <v>1.5</v>
@@ -1069,7 +1079,7 @@
         <v>46187</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C37" s="12">
         <v>1</v>
@@ -1080,25 +1090,31 @@
         <v>46187</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C38" s="12">
         <v>4</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A39" s="12"/>
-      <c r="B39" s="12"/>
-      <c r="C39" s="12"/>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A40" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="B40" s="17"/>
-      <c r="C40" s="5">
+      <c r="A39" s="19">
+        <v>46188</v>
+      </c>
+      <c r="B39" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="C39" s="20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="B42" s="17"/>
+      <c r="C42" s="5">
         <f>SUM(C3:C5)+SUM(C7:C13)+SUM(C15:C39)</f>
-        <v>79.25</v>
+        <v>81.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>